<commit_message>
Rebuilt the Resource Plan
</commit_message>
<xml_diff>
--- a/Homework 05 - Roles, Resources, Cost, and RACI.xlsx
+++ b/Homework 05 - Roles, Resources, Cost, and RACI.xlsx
@@ -8,13 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a9c7c63b8d3e1e1c/School/4 - Info Sys Proj Mgmt/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="550" documentId="11_F25DC773A252ABDACC1048EEF9187A645BDE58F3" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B92A787A-7CC4-40B5-AE8A-9C7671AA5BD8}"/>
+  <xr:revisionPtr revIDLastSave="846" documentId="11_F25DC773A252ABDACC1048EEF9187A645BDE58F3" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E60F3446-77A7-4239-B331-7B71A1FC17FB}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Roles &amp; Resources" sheetId="1" r:id="rId1"/>
-    <sheet name="Resource Plan" sheetId="2" r:id="rId2"/>
+    <sheet name="Resource Plan" sheetId="6" r:id="rId2"/>
     <sheet name="Resource &amp; Cost Plan" sheetId="3" r:id="rId3"/>
     <sheet name="Monthly Budgeted Cash Flow" sheetId="4" r:id="rId4"/>
     <sheet name="RACI Matrix" sheetId="5" r:id="rId5"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="255" uniqueCount="107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="214" uniqueCount="102">
   <si>
     <t>Role</t>
   </si>
@@ -114,21 +114,9 @@
     <t>Active Months</t>
   </si>
   <si>
-    <t>Estimated Hours</t>
-  </si>
-  <si>
     <t>Hourly Rate</t>
   </si>
   <si>
-    <t>Cost</t>
-  </si>
-  <si>
-    <t>FTE %</t>
-  </si>
-  <si>
-    <t>The resource plan estimates labor costs using a bottom-up approach based on each team member's allocation, active months, and assumed hourly rate. Resource commitments vary according to project responsibilities, with development personnel concentrated during implementation and specialized roles supporting design, integration, testing, and deployment. The estimated total labor requirement is 1,912 hours, resulting in a projected labor cost of $112,080. These estimates provide the foundation for the overall project cost plan and may be adjusted as scheduling and resource requirements are refined.</t>
-  </si>
-  <si>
     <t>Item</t>
   </si>
   <si>
@@ -138,12 +126,6 @@
     <t>Qty / Months</t>
   </si>
   <si>
-    <t>Unit Cost</t>
-  </si>
-  <si>
-    <t>Duration</t>
-  </si>
-  <si>
     <t>Total</t>
   </si>
   <si>
@@ -195,42 +177,12 @@
     <t>Operations</t>
   </si>
   <si>
-    <t>1,1912 hours</t>
-  </si>
-  <si>
-    <t>4 months</t>
-  </si>
-  <si>
-    <t>3 months</t>
-  </si>
-  <si>
-    <t>2 months</t>
-  </si>
-  <si>
     <t>One-time</t>
   </si>
   <si>
     <t>Varies</t>
   </si>
   <si>
-    <t>$300/mo</t>
-  </si>
-  <si>
-    <t>$200/mo</t>
-  </si>
-  <si>
-    <t>$150/mo</t>
-  </si>
-  <si>
-    <t>$75/mo</t>
-  </si>
-  <si>
-    <t>$100/mo</t>
-  </si>
-  <si>
-    <t>$50/mo</t>
-  </si>
-  <si>
     <t>—</t>
   </si>
   <si>
@@ -361,18 +313,49 @@
   </si>
   <si>
     <t>The RACI matrix establishes clear responsibilities and accountability across the Smart Parking Platform's major project activities. Each deliverable has one accountable team member, while responsibility for execution is distributed according to individual technical expertise. Development activities involve collaboration between backend, web, mobile, and integration personnel, while quality assurance and deployment have designated ownership. This structure supports effective coordination, reduces confusion over responsibilities, and aligns team assignments with the project's resource and communication plans.</t>
+  </si>
+  <si>
+    <t>Nov. Hrs</t>
+  </si>
+  <si>
+    <t>Oct. Hrs</t>
+  </si>
+  <si>
+    <t>Sep. Hrs</t>
+  </si>
+  <si>
+    <t>Dec. Hrs</t>
+  </si>
+  <si>
+    <t>Total Labor Cost</t>
+  </si>
+  <si>
+    <t>Total Hours</t>
+  </si>
+  <si>
+    <t>Allocation Check</t>
+  </si>
+  <si>
+    <t>Unit Cost /mo</t>
+  </si>
+  <si>
+    <t>1,192 / 4</t>
+  </si>
+  <si>
+    <t>Monthly Labor Cost</t>
+  </si>
+  <si>
+    <t>The resource plan estimates labor costs using a bottom-up approach based on each team member's allocation, active months, and assumed hourly rate. Labor hours have been distributed across September through December according to expected project activities, with development resources concentrated in October and November and specialized personnel supporting design, testing, and deployment. Monthly labor expenses are calculated directly from these allocations, providing a more accurate cash flow forecast. The total estimated labor requirement remains 1,912 hours at a projected cost of $112,080, with reconciliation checks ensuring consistency across the resource and cost plans.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="5">
+  <numFmts count="3">
     <numFmt numFmtId="6" formatCode="&quot;$&quot;#,##0_);[Red]\(&quot;$&quot;#,##0\)"/>
-    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="165" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="167" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="164" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
@@ -424,35 +407,63 @@
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="6" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="167" fontId="2" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="6" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="6" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="6" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
-    <cellStyle name="Currency" xfId="2" builtinId="4"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Percent" xfId="2" builtinId="5"/>
   </cellStyles>
-  <dxfs count="10">
+  <dxfs count="12">
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
     <dxf>
       <numFmt numFmtId="10" formatCode="&quot;$&quot;#,##0_);[Red]\(&quot;$&quot;#,##0\)"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="13" formatCode="0%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="10" formatCode="&quot;$&quot;#,##0_);[Red]\(&quot;$&quot;#,##0\)"/>
@@ -475,12 +486,6 @@
     <dxf>
       <numFmt numFmtId="10" formatCode="&quot;$&quot;#,##0_);[Red]\(&quot;$&quot;#,##0\)"/>
     </dxf>
-    <dxf>
-      <numFmt numFmtId="13" formatCode="0%"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="13" formatCode="0%"/>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -494,6 +499,10 @@
 </styleSheet>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{D938CB31-C9FB-4D58-8385-3AD410AD8CB8}" name="Table1" displayName="Table1" ref="A1:D9" totalsRowShown="0">
   <autoFilter ref="A1:D9" xr:uid="{D938CB31-C9FB-4D58-8385-3AD410AD8CB8}"/>
@@ -501,38 +510,53 @@
     <tableColumn id="1" xr3:uid="{C516ED6E-B544-4B30-80C4-8DAD7CE49AC7}" name="Role"/>
     <tableColumn id="2" xr3:uid="{45C85CE9-C9A2-4A97-B197-651EEE8CB185}" name="Name"/>
     <tableColumn id="3" xr3:uid="{CE76FF29-22C8-4516-B307-A772905AF4DC}" name="Skill Level"/>
-    <tableColumn id="4" xr3:uid="{6E9E6DBC-DDB5-4D89-92FF-58AEC1119BD0}" name="Allocation %" dataDxfId="9"/>
+    <tableColumn id="4" xr3:uid="{6E9E6DBC-DDB5-4D89-92FF-58AEC1119BD0}" name="Allocation %" dataDxfId="3" dataCellStyle="Percent"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{A1EBFA87-1A20-426C-9C2F-335605CA769B}" name="Table2" displayName="Table2" ref="A1:G10" totalsRowShown="0">
-  <autoFilter ref="A1:G10" xr:uid="{A1EBFA87-1A20-426C-9C2F-335605CA769B}"/>
-  <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{8EF702D1-ED9E-49E7-820C-351018236355}" name="Role"/>
-    <tableColumn id="2" xr3:uid="{05FBA5C4-51F7-4C32-B01C-27EA49EBCAC5}" name="Name"/>
-    <tableColumn id="3" xr3:uid="{78D8080E-F234-4688-9969-29B901A70D96}" name="FTE %" dataDxfId="8"/>
-    <tableColumn id="4" xr3:uid="{1EF63BBC-6ABE-4FC6-8B4E-3D0669D832CE}" name="Active Months"/>
-    <tableColumn id="5" xr3:uid="{0AD8CA5A-F7F1-480C-973A-E83AD4073D06}" name="Estimated Hours"/>
-    <tableColumn id="6" xr3:uid="{F7A484DB-18D2-467F-A88E-FE32B8B6B91A}" name="Hourly Rate" dataDxfId="7"/>
-    <tableColumn id="7" xr3:uid="{904B8D1B-6ACF-4CAE-9274-E87E20275BCA}" name="Cost" dataDxfId="6"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{83573F25-C56B-42D0-942B-AA570C398D1F}" name="Table7" displayName="Table7" ref="A1:K12" totalsRowShown="0">
+  <autoFilter ref="A1:K12" xr:uid="{83573F25-C56B-42D0-942B-AA570C398D1F}"/>
+  <tableColumns count="11">
+    <tableColumn id="1" xr3:uid="{482F797C-6FB3-4EA7-8CB3-534C36B73959}" name="Role">
+      <calculatedColumnFormula>'Roles &amp; Resources'!A2</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="2" xr3:uid="{A435CA4F-1E3E-43BF-8775-6714A90E6F97}" name="Name">
+      <calculatedColumnFormula>'Roles &amp; Resources'!B2</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="3" xr3:uid="{A363E3EB-C5DC-49DE-A467-76A2A8E22029}" name="Hourly Rate" dataDxfId="5"/>
+    <tableColumn id="4" xr3:uid="{95DFFD87-CB11-4380-9E56-A073B8B22C1A}" name="Sep. Hrs"/>
+    <tableColumn id="5" xr3:uid="{A9E349AF-CA26-4406-AF12-A4F9C092DA5A}" name="Oct. Hrs"/>
+    <tableColumn id="6" xr3:uid="{097587B7-2DDF-4E0C-8962-335CC9D9B42F}" name="Nov. Hrs"/>
+    <tableColumn id="7" xr3:uid="{D39B47BC-0992-4CDE-949B-E846232E3C75}" name="Dec. Hrs"/>
+    <tableColumn id="8" xr3:uid="{59E2D0B9-83D5-43D3-8068-E85CAEFF03EC}" name="Total Hours" dataDxfId="4">
+      <calculatedColumnFormula>SUM(D2:G2)</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="12" xr3:uid="{ACC25B9F-CB35-4A3D-BFA4-3786BD59BC76}" name="Active Months" dataDxfId="2">
+      <calculatedColumnFormula>COUNTIF(D2:G2, "&gt;0")</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="11" xr3:uid="{AA8D5E1F-1AB2-496D-890E-C9086C3F8B02}" name="Allocation Check" dataDxfId="0">
+      <calculatedColumnFormula>IF('Roles &amp; Resources'!D2=E25,"Yes,""No")</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="9" xr3:uid="{A9F2CD77-EEC1-4229-8010-BB2392B797A1}" name="Total Labor Cost" dataDxfId="1">
+      <calculatedColumnFormula>H2*C2</calculatedColumnFormula>
+    </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{E98EC406-D340-4D59-845B-4F16ED8D9C56}" name="Table3" displayName="Table3" ref="A1:F12" totalsRowShown="0">
-  <autoFilter ref="A1:F12" xr:uid="{E98EC406-D340-4D59-845B-4F16ED8D9C56}"/>
-  <tableColumns count="6">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{E98EC406-D340-4D59-845B-4F16ED8D9C56}" name="Table3" displayName="Table3" ref="A1:E12" totalsRowShown="0">
+  <autoFilter ref="A1:E12" xr:uid="{E98EC406-D340-4D59-845B-4F16ED8D9C56}"/>
+  <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{7AAABCCD-D02A-421B-AAC5-FA6D9F06F206}" name="Item"/>
     <tableColumn id="2" xr3:uid="{38A69F3A-DE86-498A-8B6B-0E2A36A32B61}" name="Category"/>
     <tableColumn id="3" xr3:uid="{76C20224-E494-4471-A062-9BBE5C35AF0B}" name="Qty / Months"/>
-    <tableColumn id="4" xr3:uid="{206D228E-0A36-4747-BA84-A3F93638FCC9}" name="Unit Cost"/>
-    <tableColumn id="5" xr3:uid="{1C53CEB3-CF0D-4423-9BF5-82D4AB5A21B3}" name="Duration"/>
-    <tableColumn id="6" xr3:uid="{4104E7D3-3E34-49A8-B8A3-6DACA1F5AA72}" name="Total" dataDxfId="5"/>
+    <tableColumn id="4" xr3:uid="{206D228E-0A36-4747-BA84-A3F93638FCC9}" name="Unit Cost /mo"/>
+    <tableColumn id="6" xr3:uid="{4104E7D3-3E34-49A8-B8A3-6DACA1F5AA72}" name="Total" dataDxfId="6"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium3" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -543,11 +567,11 @@
   <autoFilter ref="A1:F7" xr:uid="{57C65484-2A6E-4A35-BAD5-DE4B8CE9DD7D}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{6907FB21-04A7-40D4-95A9-332443194EE0}" name="Month"/>
-    <tableColumn id="2" xr3:uid="{3FED5E25-B6CE-43F6-B23A-939B4DBFED72}" name="Planned Labor" dataDxfId="4"/>
-    <tableColumn id="3" xr3:uid="{C7C2D9AC-CA09-47FB-9B81-1D715EF37427}" name="Planned Non-Labor" dataDxfId="3"/>
-    <tableColumn id="4" xr3:uid="{04D2F0DF-0851-49A0-AEBE-1912ACD32C2C}" name="Contingency Reserve" dataDxfId="2"/>
-    <tableColumn id="5" xr3:uid="{48F1909E-13E6-48FD-8D47-153C9018910D}" name="Total Budget" dataDxfId="1"/>
-    <tableColumn id="6" xr3:uid="{30648C0E-9875-4D54-817C-FEDD1EDE0550}" name="Cumulative Budget" dataDxfId="0"/>
+    <tableColumn id="2" xr3:uid="{3FED5E25-B6CE-43F6-B23A-939B4DBFED72}" name="Planned Labor" dataDxfId="11"/>
+    <tableColumn id="3" xr3:uid="{C7C2D9AC-CA09-47FB-9B81-1D715EF37427}" name="Planned Non-Labor" dataDxfId="10"/>
+    <tableColumn id="4" xr3:uid="{04D2F0DF-0851-49A0-AEBE-1912ACD32C2C}" name="Contingency Reserve" dataDxfId="9"/>
+    <tableColumn id="5" xr3:uid="{48F1909E-13E6-48FD-8D47-153C9018910D}" name="Total Budget" dataDxfId="8"/>
+    <tableColumn id="6" xr3:uid="{30648C0E-9875-4D54-817C-FEDD1EDE0550}" name="Cumulative Budget" dataDxfId="7"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium5" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -576,7 +600,9 @@
   <autoFilter ref="K1:L9" xr:uid="{1D4CD17C-2B93-4EE7-B9D1-EBE19683C696}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{197D5D6A-4516-4238-9271-BB871195F328}" name="Role Abbreviation"/>
-    <tableColumn id="2" xr3:uid="{5CC3F3F9-F831-47DE-B517-4D5E106F5A7C}" name="Team Member"/>
+    <tableColumn id="2" xr3:uid="{5CC3F3F9-F831-47DE-B517-4D5E106F5A7C}" name="Team Member">
+      <calculatedColumnFormula>'Roles &amp; Resources'!B2</calculatedColumnFormula>
+    </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -851,7 +877,7 @@
     <col min="1" max="1" width="37.140625" customWidth="1"/>
     <col min="2" max="2" width="24.28515625" customWidth="1"/>
     <col min="3" max="3" width="21.42578125" customWidth="1"/>
-    <col min="4" max="4" width="14.140625" customWidth="1"/>
+    <col min="4" max="4" width="14.140625" style="11" customWidth="1"/>
     <col min="6" max="6" width="82.140625" customWidth="1"/>
   </cols>
   <sheetData>
@@ -865,7 +891,7 @@
       <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="11" t="s">
         <v>3</v>
       </c>
     </row>
@@ -879,7 +905,7 @@
       <c r="C2" t="s">
         <v>20</v>
       </c>
-      <c r="D2" s="1">
+      <c r="D2" s="11">
         <v>0.5</v>
       </c>
     </row>
@@ -893,7 +919,7 @@
       <c r="C3" t="s">
         <v>20</v>
       </c>
-      <c r="D3" s="1">
+      <c r="D3" s="11">
         <v>0.75</v>
       </c>
     </row>
@@ -907,7 +933,7 @@
       <c r="C4" t="s">
         <v>21</v>
       </c>
-      <c r="D4" s="1">
+      <c r="D4" s="11">
         <v>0.75</v>
       </c>
     </row>
@@ -921,7 +947,7 @@
       <c r="C5" t="s">
         <v>21</v>
       </c>
-      <c r="D5" s="1">
+      <c r="D5" s="11">
         <v>0.75</v>
       </c>
     </row>
@@ -935,7 +961,7 @@
       <c r="C6" t="s">
         <v>21</v>
       </c>
-      <c r="D6" s="1">
+      <c r="D6" s="11">
         <v>0.5</v>
       </c>
     </row>
@@ -949,7 +975,7 @@
       <c r="C7" t="s">
         <v>20</v>
       </c>
-      <c r="D7" s="1">
+      <c r="D7" s="11">
         <v>0.5</v>
       </c>
     </row>
@@ -963,7 +989,7 @@
       <c r="C8" t="s">
         <v>21</v>
       </c>
-      <c r="D8" s="1">
+      <c r="D8" s="11">
         <v>0.5</v>
       </c>
     </row>
@@ -977,17 +1003,17 @@
       <c r="C9" t="s">
         <v>20</v>
       </c>
-      <c r="D9" s="1">
+      <c r="D9" s="11">
         <v>0.4</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="75.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="2" t="s">
+      <c r="A11" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="B11" s="2"/>
-      <c r="C11" s="2"/>
-      <c r="D11" s="2"/>
+      <c r="B11" s="7"/>
+      <c r="C11" s="7"/>
+      <c r="D11" s="7"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1001,19 +1027,18 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E588D5B2-280F-47BE-9D57-A35C525EFC7D}">
-  <dimension ref="A1:G12"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F789E40C-BD76-440A-BE6C-B1FD373E3669}">
+  <dimension ref="A1:K17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="37.140625" customWidth="1"/>
-    <col min="2" max="2" width="22.85546875" customWidth="1"/>
-    <col min="3" max="3" width="11.42578125" customWidth="1"/>
-    <col min="4" max="4" width="16" customWidth="1"/>
-    <col min="5" max="5" width="17.5703125" customWidth="1"/>
-    <col min="6" max="7" width="17.140625" customWidth="1"/>
+    <col min="2" max="2" width="24.28515625" customWidth="1"/>
+    <col min="3" max="9" width="15.7109375" customWidth="1"/>
+    <col min="10" max="10" width="15.7109375" style="9" customWidth="1"/>
+    <col min="11" max="11" width="17.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1021,248 +1046,448 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="D1" t="s">
+        <v>93</v>
+      </c>
+      <c r="E1" t="s">
+        <v>92</v>
+      </c>
+      <c r="F1" t="s">
+        <v>91</v>
+      </c>
+      <c r="G1" t="s">
+        <v>94</v>
+      </c>
+      <c r="H1" t="s">
+        <v>96</v>
+      </c>
+      <c r="I1" t="s">
         <v>23</v>
       </c>
-      <c r="E1" t="s">
-        <v>24</v>
-      </c>
-      <c r="F1" t="s">
-        <v>25</v>
-      </c>
-      <c r="G1" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+      <c r="J1" s="9" t="s">
+        <v>97</v>
+      </c>
+      <c r="K1" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A2" t="str">
+        <f>'Roles &amp; Resources'!A2</f>
+        <v>Project Manager</v>
+      </c>
+      <c r="B2" t="str">
+        <f>'Roles &amp; Resources'!B2</f>
+        <v>Alex Rivera</v>
+      </c>
+      <c r="C2" s="1">
+        <v>65</v>
+      </c>
+      <c r="D2">
+        <v>80</v>
+      </c>
+      <c r="E2">
+        <v>80</v>
+      </c>
+      <c r="F2">
+        <v>80</v>
+      </c>
+      <c r="G2">
+        <v>80</v>
+      </c>
+      <c r="H2">
+        <f t="shared" ref="H2:H8" si="0">SUM(D2:G2)</f>
+        <v>320</v>
+      </c>
+      <c r="I2">
+        <f t="shared" ref="I2:I9" si="1">COUNTIF(D2:G2, "&gt;0")</f>
         <v>4</v>
       </c>
-      <c r="B2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C2" s="1">
-        <v>0.5</v>
-      </c>
-      <c r="D2">
-        <v>4</v>
-      </c>
-      <c r="E2">
-        <f>160*C2*D2</f>
-        <v>320</v>
-      </c>
-      <c r="F2" s="3">
-        <v>65</v>
-      </c>
-      <c r="G2" s="3">
-        <f>E2*F2</f>
+      <c r="J2" s="9" t="str">
+        <f>IF('Roles &amp; Resources'!D2*I2*160=H2,"Yes", "No")</f>
+        <v>Yes</v>
+      </c>
+      <c r="K2" s="1">
+        <f>H2*C2</f>
         <v>20800</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B3" t="s">
-        <v>13</v>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A3" t="str">
+        <f>'Roles &amp; Resources'!A3</f>
+        <v>Technical Lead / Backend Developer</v>
+      </c>
+      <c r="B3" t="str">
+        <f>'Roles &amp; Resources'!B3</f>
+        <v>Charles Byrne</v>
       </c>
       <c r="C3" s="1">
-        <v>0.75</v>
+        <v>70</v>
       </c>
       <c r="D3">
+        <v>120</v>
+      </c>
+      <c r="E3">
+        <v>120</v>
+      </c>
+      <c r="F3">
+        <v>120</v>
+      </c>
+      <c r="G3">
+        <v>0</v>
+      </c>
+      <c r="H3">
+        <f t="shared" si="0"/>
+        <v>360</v>
+      </c>
+      <c r="I3">
+        <f t="shared" si="1"/>
         <v>3</v>
       </c>
-      <c r="E3">
-        <f t="shared" ref="E3:E9" si="0">160*C3*D3</f>
-        <v>360</v>
-      </c>
-      <c r="F3" s="3">
-        <v>70</v>
-      </c>
-      <c r="G3" s="3">
-        <f t="shared" ref="G3:G9" si="1">E3*F3</f>
+      <c r="J3" s="9" t="str">
+        <f>IF('Roles &amp; Resources'!D3*I3*160=H3,"Yes", "No")</f>
+        <v>Yes</v>
+      </c>
+      <c r="K3" s="1">
+        <f>H3*C3</f>
         <v>25200</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>6</v>
-      </c>
-      <c r="B4" t="s">
-        <v>14</v>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A4" t="str">
+        <f>'Roles &amp; Resources'!A4</f>
+        <v>Frontend / Web Developer</v>
+      </c>
+      <c r="B4" t="str">
+        <f>'Roles &amp; Resources'!B4</f>
+        <v>Taylor Pearce</v>
       </c>
       <c r="C4" s="1">
-        <v>0.75</v>
+        <v>50</v>
       </c>
       <c r="D4">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E4">
+        <v>120</v>
+      </c>
+      <c r="F4">
+        <v>120</v>
+      </c>
+      <c r="G4">
+        <v>0</v>
+      </c>
+      <c r="H4">
         <f t="shared" si="0"/>
         <v>240</v>
       </c>
-      <c r="F4" s="3">
-        <v>50</v>
-      </c>
-      <c r="G4" s="3">
+      <c r="I4">
         <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="J4" s="9" t="str">
+        <f>IF('Roles &amp; Resources'!D4*I4*160=H4,"Yes", "No")</f>
+        <v>Yes</v>
+      </c>
+      <c r="K4" s="1">
+        <f>H4*C4</f>
         <v>12000</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>7</v>
-      </c>
-      <c r="B5" t="s">
-        <v>17</v>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A5" t="str">
+        <f>'Roles &amp; Resources'!A5</f>
+        <v>Mobile Developer</v>
+      </c>
+      <c r="B5" t="str">
+        <f>'Roles &amp; Resources'!B5</f>
+        <v>Brittany Nguyen</v>
       </c>
       <c r="C5" s="1">
-        <v>0.75</v>
+        <v>55</v>
       </c>
       <c r="D5">
+        <v>0</v>
+      </c>
+      <c r="E5">
+        <v>120</v>
+      </c>
+      <c r="F5">
+        <v>120</v>
+      </c>
+      <c r="G5">
+        <v>0</v>
+      </c>
+      <c r="H5">
+        <f>SUM(D5:G5)</f>
+        <v>240</v>
+      </c>
+      <c r="I5">
+        <f t="shared" si="1"/>
         <v>2</v>
       </c>
-      <c r="E5">
+      <c r="J5" s="9" t="str">
+        <f>IF('Roles &amp; Resources'!D5*I5*160=H5,"Yes", "No")</f>
+        <v>Yes</v>
+      </c>
+      <c r="K5" s="1">
+        <f>H5*C5</f>
+        <v>13200</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A6" t="str">
+        <f>'Roles &amp; Resources'!A6</f>
+        <v>UI/UX Designer</v>
+      </c>
+      <c r="B6" t="str">
+        <f>'Roles &amp; Resources'!B6</f>
+        <v>Lexi Harper</v>
+      </c>
+      <c r="C6" s="1">
+        <v>45</v>
+      </c>
+      <c r="D6">
+        <v>80</v>
+      </c>
+      <c r="E6">
+        <v>80</v>
+      </c>
+      <c r="F6">
+        <v>0</v>
+      </c>
+      <c r="G6">
+        <v>0</v>
+      </c>
+      <c r="H6">
+        <f t="shared" si="0"/>
+        <v>160</v>
+      </c>
+      <c r="I6">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="J6" s="9" t="str">
+        <f>IF('Roles &amp; Resources'!D6*I6*160=H6,"Yes", "No")</f>
+        <v>Yes</v>
+      </c>
+      <c r="K6" s="1">
+        <f>H6*C6</f>
+        <v>7200</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A7" t="str">
+        <f>'Roles &amp; Resources'!A7</f>
+        <v>Integration Developer</v>
+      </c>
+      <c r="B7" t="str">
+        <f>'Roles &amp; Resources'!B7</f>
+        <v>William Cooke</v>
+      </c>
+      <c r="C7" s="1">
+        <v>65</v>
+      </c>
+      <c r="D7">
+        <v>0</v>
+      </c>
+      <c r="E7">
+        <v>80</v>
+      </c>
+      <c r="F7">
+        <v>80</v>
+      </c>
+      <c r="G7">
+        <v>0</v>
+      </c>
+      <c r="H7">
+        <f t="shared" si="0"/>
+        <v>160</v>
+      </c>
+      <c r="I7">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="J7" s="9" t="str">
+        <f>IF('Roles &amp; Resources'!D7*I7*160=H7,"Yes", "No")</f>
+        <v>Yes</v>
+      </c>
+      <c r="K7" s="1">
+        <f>H7*C7</f>
+        <v>10400</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A8" t="str">
+        <f>'Roles &amp; Resources'!A8</f>
+        <v>QA Tester</v>
+      </c>
+      <c r="B8" t="str">
+        <f>'Roles &amp; Resources'!B8</f>
+        <v>Ayden Moss</v>
+      </c>
+      <c r="C8" s="1">
+        <v>45</v>
+      </c>
+      <c r="D8">
+        <v>0</v>
+      </c>
+      <c r="E8">
+        <v>80</v>
+      </c>
+      <c r="F8">
+        <v>80</v>
+      </c>
+      <c r="G8">
+        <v>80</v>
+      </c>
+      <c r="H8">
         <f t="shared" si="0"/>
         <v>240</v>
       </c>
-      <c r="F5" s="3">
-        <v>55</v>
-      </c>
-      <c r="G5" s="3">
+      <c r="I8">
         <f t="shared" si="1"/>
-        <v>13200</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>8</v>
-      </c>
-      <c r="B6" t="s">
-        <v>16</v>
-      </c>
-      <c r="C6" s="1">
-        <v>0.5</v>
-      </c>
-      <c r="D6">
-        <v>2</v>
-      </c>
-      <c r="E6">
-        <f t="shared" si="0"/>
-        <v>160</v>
-      </c>
-      <c r="F6" s="3">
-        <v>45</v>
-      </c>
-      <c r="G6" s="3">
+        <v>3</v>
+      </c>
+      <c r="J8" s="9" t="str">
+        <f>IF('Roles &amp; Resources'!D8*I8*160=H8,"Yes", "No")</f>
+        <v>Yes</v>
+      </c>
+      <c r="K8" s="1">
+        <f>H8*C8</f>
+        <v>10800</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A9" t="str">
+        <f>'Roles &amp; Resources'!A9</f>
+        <v>DevOps / Database Engineer</v>
+      </c>
+      <c r="B9" t="str">
+        <f>'Roles &amp; Resources'!B9</f>
+        <v>Paige Hoffman</v>
+      </c>
+      <c r="C9" s="1">
+        <v>65</v>
+      </c>
+      <c r="D9">
+        <v>64</v>
+      </c>
+      <c r="E9">
+        <v>0</v>
+      </c>
+      <c r="F9">
+        <v>64</v>
+      </c>
+      <c r="G9">
+        <v>64</v>
+      </c>
+      <c r="H9">
+        <f>SUM(D9:G9)</f>
+        <v>192</v>
+      </c>
+      <c r="I9">
         <f t="shared" si="1"/>
-        <v>7200</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>9</v>
-      </c>
-      <c r="B7" t="s">
-        <v>19</v>
-      </c>
-      <c r="C7" s="1">
-        <v>0.5</v>
-      </c>
-      <c r="D7">
-        <v>2</v>
-      </c>
-      <c r="E7">
-        <f t="shared" si="0"/>
-        <v>160</v>
-      </c>
-      <c r="F7" s="3">
-        <v>65</v>
-      </c>
-      <c r="G7" s="3">
-        <f t="shared" si="1"/>
-        <v>10400</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>10</v>
-      </c>
-      <c r="B8" t="s">
-        <v>15</v>
-      </c>
-      <c r="C8" s="1">
-        <v>0.5</v>
-      </c>
-      <c r="D8">
         <v>3</v>
       </c>
-      <c r="E8">
-        <f t="shared" si="0"/>
-        <v>240</v>
-      </c>
-      <c r="F8" s="3">
-        <v>45</v>
-      </c>
-      <c r="G8" s="3">
-        <f t="shared" si="1"/>
-        <v>10800</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>11</v>
-      </c>
-      <c r="B9" t="s">
-        <v>18</v>
-      </c>
-      <c r="C9" s="1">
-        <v>0.4</v>
-      </c>
-      <c r="D9">
-        <v>3</v>
-      </c>
-      <c r="E9">
-        <f t="shared" si="0"/>
-        <v>192</v>
-      </c>
-      <c r="F9" s="3">
-        <v>65</v>
-      </c>
-      <c r="G9" s="3">
-        <f t="shared" si="1"/>
+      <c r="J9" s="9" t="str">
+        <f>IF('Roles &amp; Resources'!D9*I9*160=H9,"Yes", "No")</f>
+        <v>Yes</v>
+      </c>
+      <c r="K9" s="1">
+        <f>H9*C9</f>
         <v>12480</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="E10" s="5">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A10" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="B10" s="2"/>
+      <c r="C10" s="5"/>
+      <c r="D10" s="2">
+        <f>SUM(D2:D9)</f>
+        <v>344</v>
+      </c>
+      <c r="E10" s="2">
         <f>SUM(E2:E9)</f>
+        <v>680</v>
+      </c>
+      <c r="F10" s="2">
+        <f>SUM(F2:F9)</f>
+        <v>664</v>
+      </c>
+      <c r="G10" s="2">
+        <f>SUM(G2:G9)</f>
+        <v>224</v>
+      </c>
+      <c r="H10" s="3">
+        <f>SUM(H2:H9)</f>
         <v>1912</v>
       </c>
-      <c r="G10" s="6">
-        <f>SUM(G2:G9)</f>
+      <c r="I10" s="3"/>
+      <c r="J10" s="13"/>
+      <c r="K10" s="5">
+        <f>IF(SUM(K2:K9)=SUM(D12:G12),SUM(D12:G12),"Mismatch")</f>
         <v>112080</v>
       </c>
     </row>
-    <row r="12" spans="1:7" ht="63.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="B12" s="2"/>
-      <c r="C12" s="2"/>
-      <c r="D12" s="2"/>
-      <c r="E12" s="2"/>
-      <c r="F12" s="2"/>
-      <c r="G12" s="2"/>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="C11" s="1"/>
+      <c r="H11" s="8"/>
+      <c r="I11" s="8"/>
+      <c r="J11" s="15"/>
+      <c r="K11" s="1"/>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>100</v>
+      </c>
+      <c r="C12" s="1"/>
+      <c r="D12" s="1">
+        <f>(C2*D2)+(C3*D3)+(C4*D4)+(C5*D5)+(C6*D6)+(C7*D7)+(C8*D8)+(C9*D9)</f>
+        <v>21360</v>
+      </c>
+      <c r="E12" s="1">
+        <f>(C2*E2)+(C3*E3)+(C4*E4)+(C5*E5)+(C6*E6)+(C7*E7)+(C8*E8)+(C9*E9)</f>
+        <v>38600</v>
+      </c>
+      <c r="F12" s="1">
+        <f>(C2*F2)+(C3*F3)+(C4*F4)+(C5*F5)+(C6*F6)+(C7*F7)+(C8*F8)+(C9*F9)</f>
+        <v>39160</v>
+      </c>
+      <c r="G12" s="1">
+        <f>(C2*G2)+(C3*G3)+(C4*G4)+(C5*G5)+(C6*G6)+(C7*G7)+(C8*G8)+(C9*G9)</f>
+        <v>12960</v>
+      </c>
+      <c r="H12" s="8"/>
+      <c r="I12" s="8"/>
+      <c r="J12" s="15"/>
+      <c r="K12" s="1"/>
+    </row>
+    <row r="14" spans="1:11" ht="63.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="B14" s="7"/>
+      <c r="C14" s="7"/>
+      <c r="D14" s="7"/>
+      <c r="E14" s="7"/>
+      <c r="F14" s="7"/>
+      <c r="G14" s="7"/>
+      <c r="H14" s="7"/>
+      <c r="I14" s="7"/>
+      <c r="J14" s="7"/>
+      <c r="K14" s="7"/>
+    </row>
+    <row r="17" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B17" s="12"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A12:G12"/>
+    <mergeCell ref="A14:K14"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
@@ -1273,243 +1498,223 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{37832EDD-D42C-4B3B-8480-EE395C5A64E2}">
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="37.140625" customWidth="1"/>
     <col min="2" max="2" width="20" customWidth="1"/>
-    <col min="3" max="6" width="17.140625" customWidth="1"/>
+    <col min="3" max="5" width="17.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" t="s">
+        <v>98</v>
+      </c>
+      <c r="E1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>29</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B2" t="s">
+        <v>39</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="D2" t="s">
+        <v>46</v>
+      </c>
+      <c r="E2" s="1">
+        <f>'Resource Plan'!K10</f>
+        <v>112080</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>30</v>
       </c>
-      <c r="C1" t="s">
+      <c r="B3" t="s">
+        <v>40</v>
+      </c>
+      <c r="C3">
+        <v>4</v>
+      </c>
+      <c r="D3" s="1">
+        <v>300</v>
+      </c>
+      <c r="E3" s="1">
+        <f>C3*D3</f>
+        <v>1200</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
         <v>31</v>
       </c>
-      <c r="D1" t="s">
+      <c r="B4" t="s">
+        <v>41</v>
+      </c>
+      <c r="C4">
+        <v>3</v>
+      </c>
+      <c r="D4" s="1">
+        <v>200</v>
+      </c>
+      <c r="E4" s="1">
+        <f t="shared" ref="E4:E8" si="0">C4*D4</f>
+        <v>600</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
         <v>32</v>
       </c>
-      <c r="E1" t="s">
+      <c r="B5" t="s">
+        <v>41</v>
+      </c>
+      <c r="C5">
+        <v>2</v>
+      </c>
+      <c r="D5" s="1">
+        <v>150</v>
+      </c>
+      <c r="E5" s="1">
+        <f t="shared" si="0"/>
+        <v>300</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
         <v>33</v>
       </c>
-      <c r="F1" t="s">
+      <c r="B6" t="s">
+        <v>42</v>
+      </c>
+      <c r="C6">
+        <v>2</v>
+      </c>
+      <c r="D6" s="1">
+        <v>75</v>
+      </c>
+      <c r="E6" s="1">
+        <f t="shared" si="0"/>
+        <v>150</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>43</v>
+      </c>
+      <c r="B7" t="s">
+        <v>42</v>
+      </c>
+      <c r="C7">
+        <v>3</v>
+      </c>
+      <c r="D7" s="1">
+        <v>100</v>
+      </c>
+      <c r="E7" s="1">
+        <f t="shared" si="0"/>
+        <v>300</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+      <c r="B8" t="s">
+        <v>42</v>
+      </c>
+      <c r="C8">
+        <v>4</v>
+      </c>
+      <c r="D8" s="1">
+        <v>50</v>
+      </c>
+      <c r="E8" s="1">
+        <f t="shared" si="0"/>
+        <v>200</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
         <v>35</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B9" t="s">
+        <v>44</v>
+      </c>
+      <c r="C9" t="s">
         <v>45</v>
       </c>
-      <c r="C2" t="s">
-        <v>51</v>
-      </c>
-      <c r="D2" t="s">
-        <v>56</v>
-      </c>
-      <c r="E2" t="s">
-        <v>52</v>
-      </c>
-      <c r="F2" s="3">
-        <v>112080</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+      <c r="D9" s="14">
+        <v>1000</v>
+      </c>
+      <c r="E9" s="1">
+        <f>D9</f>
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
         <v>36</v>
       </c>
-      <c r="B3" t="s">
-        <v>46</v>
-      </c>
-      <c r="C3" t="s">
-        <v>52</v>
-      </c>
-      <c r="D3" t="s">
-        <v>57</v>
-      </c>
-      <c r="E3" t="s">
-        <v>52</v>
-      </c>
-      <c r="F3" s="3">
-        <v>1200</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+      <c r="E10" s="1">
+        <f>SUM(E2:E9)</f>
+        <v>115830</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
         <v>37</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B11" t="s">
+        <v>48</v>
+      </c>
+      <c r="C11" s="4">
+        <v>0.1</v>
+      </c>
+      <c r="D11" t="s">
         <v>47</v>
       </c>
-      <c r="C4" t="s">
-        <v>53</v>
-      </c>
-      <c r="D4" t="s">
-        <v>58</v>
-      </c>
-      <c r="E4" t="s">
-        <v>53</v>
-      </c>
-      <c r="F4" s="3">
-        <v>600</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+      <c r="E11" s="1">
+        <f>E10*C11</f>
+        <v>11583</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="B5" t="s">
-        <v>47</v>
-      </c>
-      <c r="C5" t="s">
-        <v>54</v>
-      </c>
-      <c r="D5" t="s">
-        <v>59</v>
-      </c>
-      <c r="E5" t="s">
-        <v>54</v>
-      </c>
-      <c r="F5" s="3">
-        <v>300</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>39</v>
-      </c>
-      <c r="B6" t="s">
-        <v>48</v>
-      </c>
-      <c r="C6" t="s">
-        <v>54</v>
-      </c>
-      <c r="D6" t="s">
-        <v>60</v>
-      </c>
-      <c r="E6" t="s">
-        <v>54</v>
-      </c>
-      <c r="F6" s="3">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
+      <c r="E12" s="5">
+        <f>SUM(E10:E11)</f>
+        <v>127413</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" ht="93.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="B7" t="s">
-        <v>48</v>
-      </c>
-      <c r="C7" t="s">
-        <v>53</v>
-      </c>
-      <c r="D7" t="s">
-        <v>61</v>
-      </c>
-      <c r="E7" t="s">
-        <v>53</v>
-      </c>
-      <c r="F7" s="3">
-        <v>300</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>40</v>
-      </c>
-      <c r="B8" t="s">
-        <v>48</v>
-      </c>
-      <c r="C8" t="s">
-        <v>52</v>
-      </c>
-      <c r="D8" t="s">
-        <v>62</v>
-      </c>
-      <c r="E8" t="s">
-        <v>52</v>
-      </c>
-      <c r="F8" s="3">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>41</v>
-      </c>
-      <c r="B9" t="s">
-        <v>50</v>
-      </c>
-      <c r="C9" t="s">
-        <v>55</v>
-      </c>
-      <c r="D9" s="7">
-        <v>1000</v>
-      </c>
-      <c r="E9" s="8" t="s">
-        <v>63</v>
-      </c>
-      <c r="F9" s="3">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>42</v>
-      </c>
-      <c r="F10" s="3">
-        <v>115830</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>43</v>
-      </c>
-      <c r="B11" t="s">
-        <v>64</v>
-      </c>
-      <c r="C11" s="9">
-        <v>0.1</v>
-      </c>
-      <c r="D11" s="8" t="s">
-        <v>63</v>
-      </c>
-      <c r="E11" s="8" t="s">
-        <v>63</v>
-      </c>
-      <c r="F11" s="3">
-        <v>11583</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A12" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="F12" s="10">
-        <v>127413</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" ht="75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="B14" s="2"/>
-      <c r="C14" s="2"/>
-      <c r="D14" s="2"/>
-      <c r="E14" s="2"/>
-      <c r="F14" s="2"/>
+      <c r="B14" s="7"/>
+      <c r="C14" s="7"/>
+      <c r="D14" s="7"/>
+      <c r="E14" s="7"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A14:F14"/>
+    <mergeCell ref="A14:E14"/>
   </mergeCells>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1534,167 +1739,173 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>66</v>
+        <v>50</v>
       </c>
       <c r="B1" t="s">
-        <v>67</v>
+        <v>51</v>
       </c>
       <c r="C1" t="s">
-        <v>68</v>
+        <v>52</v>
       </c>
       <c r="D1" t="s">
-        <v>69</v>
+        <v>53</v>
       </c>
       <c r="E1" t="s">
-        <v>70</v>
+        <v>54</v>
       </c>
       <c r="F1" t="s">
-        <v>71</v>
+        <v>55</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>72</v>
-      </c>
-      <c r="B2" s="3">
-        <v>22000</v>
-      </c>
-      <c r="C2" s="3">
-        <v>450</v>
-      </c>
-      <c r="D2" s="3">
+        <v>56</v>
+      </c>
+      <c r="B2" s="1">
+        <f>'Resource Plan'!D12</f>
+        <v>21360</v>
+      </c>
+      <c r="C2" s="1">
+        <v>426</v>
+      </c>
+      <c r="D2" s="1">
         <v>0</v>
       </c>
-      <c r="E2" s="3">
+      <c r="E2" s="1">
         <f>SUM(B2:D2)</f>
-        <v>22450</v>
-      </c>
-      <c r="F2" s="3">
+        <v>21786</v>
+      </c>
+      <c r="F2" s="1">
         <f>SUM($E$2:E2)</f>
-        <v>22450</v>
+        <v>21786</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>73</v>
-      </c>
-      <c r="B3" s="3">
-        <v>40000</v>
-      </c>
-      <c r="C3" s="3">
-        <v>1050</v>
-      </c>
-      <c r="D3" s="3">
+        <v>57</v>
+      </c>
+      <c r="B3" s="1">
+        <f>'Resource Plan'!E12</f>
+        <v>38600</v>
+      </c>
+      <c r="C3" s="1">
+        <v>874</v>
+      </c>
+      <c r="D3" s="1">
         <v>0</v>
       </c>
-      <c r="E3" s="3">
-        <f t="shared" ref="E3:E6" si="0">SUM(B3:D3)</f>
-        <v>41050</v>
-      </c>
-      <c r="F3" s="3">
+      <c r="E3" s="1">
+        <f t="shared" ref="E3:E5" si="0">SUM(B3:D3)</f>
+        <v>39474</v>
+      </c>
+      <c r="F3" s="1">
         <f>SUM($E$2:E3)</f>
-        <v>63500</v>
+        <v>61260</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>74</v>
-      </c>
-      <c r="B4" s="3">
-        <v>36000</v>
-      </c>
-      <c r="C4" s="3">
-        <v>1150</v>
-      </c>
-      <c r="D4" s="3">
+        <v>58</v>
+      </c>
+      <c r="B4" s="1">
+        <f>'Resource Plan'!F12</f>
+        <v>39160</v>
+      </c>
+      <c r="C4" s="1">
+        <v>800</v>
+      </c>
+      <c r="D4" s="1">
         <v>0</v>
       </c>
-      <c r="E4" s="3">
+      <c r="E4" s="1">
         <f t="shared" si="0"/>
-        <v>37150</v>
-      </c>
-      <c r="F4" s="3">
+        <v>39960</v>
+      </c>
+      <c r="F4" s="1">
         <f>SUM($E$2:E4)</f>
-        <v>100650</v>
+        <v>101220</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>75</v>
-      </c>
-      <c r="B5" s="3">
-        <v>14080</v>
-      </c>
-      <c r="C5" s="3">
-        <v>1100</v>
-      </c>
-      <c r="D5" s="3">
+        <v>59</v>
+      </c>
+      <c r="B5" s="1">
+        <f>'Resource Plan'!G12</f>
+        <v>12960</v>
+      </c>
+      <c r="C5" s="1">
+        <v>1650</v>
+      </c>
+      <c r="D5" s="1">
         <v>0</v>
       </c>
-      <c r="E5" s="3">
+      <c r="E5" s="1">
         <f t="shared" si="0"/>
-        <v>15180</v>
-      </c>
-      <c r="F5" s="3">
+        <v>14610</v>
+      </c>
+      <c r="F5" s="1">
         <f>SUM($E$2:E5)</f>
         <v>115830</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>76</v>
-      </c>
-      <c r="B6" s="3">
+        <v>60</v>
+      </c>
+      <c r="B6" s="1">
         <v>0</v>
       </c>
-      <c r="C6" s="3">
+      <c r="C6" s="1">
         <v>0</v>
       </c>
-      <c r="D6" s="3">
+      <c r="D6" s="1">
+        <f>'Resource &amp; Cost Plan'!E11</f>
         <v>11583</v>
       </c>
-      <c r="E6" s="3">
-        <f t="shared" si="0"/>
+      <c r="E6" s="1">
+        <f>SUM(B6:D6)</f>
         <v>11583</v>
       </c>
-      <c r="F6" s="3">
+      <c r="F6" s="1">
         <f>SUM($E$2:E6)</f>
         <v>127413</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="B7" s="10">
-        <f>SUM(B2:B6)</f>
+      <c r="A7" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B7" s="5">
+        <f>IF(SUM(B2:B6)='Resource Plan'!K10,SUM(B2:B6),"Mismatch")</f>
         <v>112080</v>
       </c>
-      <c r="C7" s="10">
+      <c r="C7" s="5">
         <f>SUM(C2:C6)</f>
         <v>3750</v>
       </c>
-      <c r="D7" s="10">
+      <c r="D7" s="5">
         <f>SUM(D2:D6)</f>
         <v>11583</v>
       </c>
-      <c r="E7" s="10">
-        <f>SUM(E2:E6)</f>
+      <c r="E7" s="5">
+        <f>IF(SUM(E2:E6)='Resource &amp; Cost Plan'!E12,SUM(E2:E6),"Mismatch")</f>
         <v>127413</v>
       </c>
-      <c r="F7" s="10">
+      <c r="F7" s="5">
+        <f>E7</f>
         <v>127413</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="63.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="B9" s="2"/>
-      <c r="C9" s="2"/>
-      <c r="D9" s="2"/>
-      <c r="E9" s="2"/>
-      <c r="F9" s="2"/>
+      <c r="A9" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="B9" s="7"/>
+      <c r="C9" s="7"/>
+      <c r="D9" s="7"/>
+      <c r="E9" s="7"/>
+      <c r="F9" s="7"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1719,447 +1930,455 @@
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>78</v>
+        <v>62</v>
       </c>
       <c r="B1" t="s">
-        <v>79</v>
+        <v>63</v>
       </c>
       <c r="C1" t="s">
-        <v>80</v>
+        <v>64</v>
       </c>
       <c r="D1" t="s">
-        <v>81</v>
+        <v>65</v>
       </c>
       <c r="E1" t="s">
-        <v>82</v>
+        <v>66</v>
       </c>
       <c r="F1" t="s">
-        <v>83</v>
+        <v>67</v>
       </c>
       <c r="G1" t="s">
-        <v>84</v>
+        <v>68</v>
       </c>
       <c r="H1" t="s">
-        <v>85</v>
+        <v>69</v>
       </c>
       <c r="I1" t="s">
-        <v>86</v>
+        <v>70</v>
       </c>
       <c r="K1" t="s">
-        <v>87</v>
+        <v>71</v>
       </c>
       <c r="L1" t="s">
-        <v>88</v>
+        <v>72</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>89</v>
+        <v>73</v>
       </c>
       <c r="B2" t="s">
-        <v>101</v>
+        <v>85</v>
       </c>
       <c r="C2" t="s">
-        <v>102</v>
+        <v>86</v>
       </c>
       <c r="D2" t="s">
-        <v>103</v>
+        <v>87</v>
       </c>
       <c r="E2" t="s">
-        <v>103</v>
+        <v>87</v>
       </c>
       <c r="F2" t="s">
-        <v>104</v>
+        <v>88</v>
       </c>
       <c r="G2" t="s">
-        <v>102</v>
+        <v>86</v>
       </c>
       <c r="H2" t="s">
-        <v>102</v>
+        <v>86</v>
       </c>
       <c r="I2" t="s">
-        <v>103</v>
+        <v>87</v>
       </c>
       <c r="K2" t="s">
-        <v>79</v>
-      </c>
-      <c r="L2" t="s">
-        <v>12</v>
+        <v>63</v>
+      </c>
+      <c r="L2" t="str">
+        <f>'Roles &amp; Resources'!B2</f>
+        <v>Alex Rivera</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>90</v>
+        <v>74</v>
       </c>
       <c r="B3" t="s">
-        <v>102</v>
+        <v>86</v>
       </c>
       <c r="C3" t="s">
-        <v>101</v>
+        <v>85</v>
       </c>
       <c r="D3" t="s">
-        <v>102</v>
+        <v>86</v>
       </c>
       <c r="E3" t="s">
-        <v>102</v>
+        <v>86</v>
       </c>
       <c r="F3" t="s">
-        <v>103</v>
+        <v>87</v>
       </c>
       <c r="G3" t="s">
-        <v>104</v>
+        <v>88</v>
       </c>
       <c r="H3" t="s">
-        <v>102</v>
+        <v>86</v>
       </c>
       <c r="I3" t="s">
-        <v>104</v>
+        <v>88</v>
       </c>
       <c r="K3" t="s">
-        <v>80</v>
-      </c>
-      <c r="L3" t="s">
-        <v>13</v>
+        <v>64</v>
+      </c>
+      <c r="L3" t="str">
+        <f>'Roles &amp; Resources'!B3</f>
+        <v>Charles Byrne</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>91</v>
+        <v>75</v>
       </c>
       <c r="B4" t="s">
-        <v>103</v>
+        <v>87</v>
       </c>
       <c r="C4" t="s">
-        <v>102</v>
+        <v>86</v>
       </c>
       <c r="D4" t="s">
-        <v>104</v>
+        <v>88</v>
       </c>
       <c r="E4" t="s">
-        <v>104</v>
+        <v>88</v>
       </c>
       <c r="F4" t="s">
-        <v>101</v>
+        <v>85</v>
       </c>
       <c r="G4" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="H4" t="s">
-        <v>102</v>
+        <v>86</v>
       </c>
       <c r="I4" t="s">
-        <v>103</v>
+        <v>87</v>
       </c>
       <c r="K4" t="s">
-        <v>81</v>
-      </c>
-      <c r="L4" t="s">
-        <v>14</v>
+        <v>65</v>
+      </c>
+      <c r="L4" t="str">
+        <f>'Roles &amp; Resources'!B4</f>
+        <v>Taylor Pearce</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>92</v>
+        <v>76</v>
       </c>
       <c r="B5" t="s">
-        <v>103</v>
+        <v>87</v>
       </c>
       <c r="C5" t="s">
-        <v>101</v>
+        <v>85</v>
       </c>
       <c r="D5" t="s">
-        <v>104</v>
+        <v>88</v>
       </c>
       <c r="E5" t="s">
-        <v>104</v>
+        <v>88</v>
       </c>
       <c r="F5" t="s">
-        <v>102</v>
+        <v>86</v>
       </c>
       <c r="G5" t="s">
-        <v>102</v>
+        <v>86</v>
       </c>
       <c r="H5" t="s">
-        <v>102</v>
+        <v>86</v>
       </c>
       <c r="I5" t="s">
-        <v>102</v>
+        <v>86</v>
       </c>
       <c r="K5" t="s">
-        <v>82</v>
-      </c>
-      <c r="L5" t="s">
-        <v>17</v>
+        <v>66</v>
+      </c>
+      <c r="L5" t="str">
+        <f>'Roles &amp; Resources'!B5</f>
+        <v>Brittany Nguyen</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>93</v>
+        <v>77</v>
       </c>
       <c r="B6" t="s">
-        <v>103</v>
+        <v>87</v>
       </c>
       <c r="C6" t="s">
-        <v>101</v>
+        <v>85</v>
       </c>
       <c r="D6" t="s">
-        <v>104</v>
+        <v>88</v>
       </c>
       <c r="E6" t="s">
-        <v>104</v>
+        <v>88</v>
       </c>
       <c r="F6" t="s">
-        <v>102</v>
+        <v>86</v>
       </c>
       <c r="G6" t="s">
-        <v>104</v>
+        <v>88</v>
       </c>
       <c r="H6" t="s">
-        <v>102</v>
+        <v>86</v>
       </c>
       <c r="I6" t="s">
-        <v>104</v>
+        <v>88</v>
       </c>
       <c r="K6" t="s">
-        <v>83</v>
-      </c>
-      <c r="L6" t="s">
-        <v>16</v>
+        <v>67</v>
+      </c>
+      <c r="L6" t="str">
+        <f>'Roles &amp; Resources'!B6</f>
+        <v>Lexi Harper</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>94</v>
+        <v>78</v>
       </c>
       <c r="B7" t="s">
-        <v>103</v>
+        <v>87</v>
       </c>
       <c r="C7" t="s">
-        <v>105</v>
+        <v>89</v>
       </c>
       <c r="D7" t="s">
-        <v>104</v>
+        <v>88</v>
       </c>
       <c r="E7" t="s">
-        <v>104</v>
+        <v>88</v>
       </c>
       <c r="F7" t="s">
-        <v>102</v>
+        <v>86</v>
       </c>
       <c r="G7" t="s">
-        <v>104</v>
+        <v>88</v>
       </c>
       <c r="H7" t="s">
-        <v>102</v>
+        <v>86</v>
       </c>
       <c r="I7" t="s">
-        <v>102</v>
+        <v>86</v>
       </c>
       <c r="K7" t="s">
-        <v>84</v>
-      </c>
-      <c r="L7" t="s">
-        <v>19</v>
+        <v>68</v>
+      </c>
+      <c r="L7" t="str">
+        <f>'Roles &amp; Resources'!B7</f>
+        <v>William Cooke</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>95</v>
+        <v>79</v>
       </c>
       <c r="B8" t="s">
-        <v>103</v>
+        <v>87</v>
       </c>
       <c r="C8" t="s">
-        <v>105</v>
+        <v>89</v>
       </c>
       <c r="D8" t="s">
-        <v>104</v>
+        <v>88</v>
       </c>
       <c r="E8" t="s">
-        <v>104</v>
+        <v>88</v>
       </c>
       <c r="F8" t="s">
-        <v>102</v>
+        <v>86</v>
       </c>
       <c r="G8" t="s">
-        <v>104</v>
+        <v>88</v>
       </c>
       <c r="H8" t="s">
-        <v>102</v>
+        <v>86</v>
       </c>
       <c r="I8" t="s">
-        <v>102</v>
+        <v>86</v>
       </c>
       <c r="K8" t="s">
-        <v>85</v>
-      </c>
-      <c r="L8" t="s">
-        <v>15</v>
+        <v>69</v>
+      </c>
+      <c r="L8" t="str">
+        <f>'Roles &amp; Resources'!B8</f>
+        <v>Ayden Moss</v>
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>96</v>
+        <v>80</v>
       </c>
       <c r="B9" t="s">
-        <v>103</v>
+        <v>87</v>
       </c>
       <c r="C9" t="s">
-        <v>105</v>
+        <v>89</v>
       </c>
       <c r="D9" t="s">
-        <v>104</v>
+        <v>88</v>
       </c>
       <c r="E9" t="s">
-        <v>102</v>
+        <v>86</v>
       </c>
       <c r="F9" t="s">
-        <v>104</v>
+        <v>88</v>
       </c>
       <c r="G9" t="s">
-        <v>102</v>
+        <v>86</v>
       </c>
       <c r="H9" t="s">
-        <v>102</v>
+        <v>86</v>
       </c>
       <c r="I9" t="s">
-        <v>104</v>
+        <v>88</v>
       </c>
       <c r="K9" t="s">
-        <v>86</v>
-      </c>
-      <c r="L9" t="s">
-        <v>18</v>
+        <v>70</v>
+      </c>
+      <c r="L9" t="str">
+        <f>'Roles &amp; Resources'!B9</f>
+        <v>Paige Hoffman</v>
       </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>97</v>
+        <v>81</v>
       </c>
       <c r="B10" t="s">
-        <v>103</v>
+        <v>87</v>
       </c>
       <c r="C10" t="s">
-        <v>102</v>
+        <v>86</v>
       </c>
       <c r="D10" t="s">
-        <v>104</v>
+        <v>88</v>
       </c>
       <c r="E10" t="s">
-        <v>104</v>
+        <v>88</v>
       </c>
       <c r="F10" t="s">
-        <v>103</v>
+        <v>87</v>
       </c>
       <c r="G10" t="s">
-        <v>104</v>
+        <v>88</v>
       </c>
       <c r="H10" t="s">
-        <v>101</v>
+        <v>85</v>
       </c>
       <c r="I10" t="s">
-        <v>102</v>
+        <v>86</v>
       </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>98</v>
+        <v>82</v>
       </c>
       <c r="B11" t="s">
-        <v>103</v>
+        <v>87</v>
       </c>
       <c r="C11" t="s">
-        <v>102</v>
+        <v>86</v>
       </c>
       <c r="D11" t="s">
-        <v>102</v>
+        <v>86</v>
       </c>
       <c r="E11" t="s">
-        <v>102</v>
+        <v>86</v>
       </c>
       <c r="F11" t="s">
-        <v>102</v>
+        <v>86</v>
       </c>
       <c r="G11" t="s">
-        <v>102</v>
+        <v>86</v>
       </c>
       <c r="H11" t="s">
-        <v>101</v>
+        <v>85</v>
       </c>
       <c r="I11" t="s">
-        <v>103</v>
+        <v>87</v>
       </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>99</v>
+        <v>83</v>
       </c>
       <c r="B12" t="s">
-        <v>102</v>
+        <v>86</v>
       </c>
       <c r="C12" t="s">
-        <v>104</v>
+        <v>88</v>
       </c>
       <c r="D12" t="s">
-        <v>102</v>
+        <v>86</v>
       </c>
       <c r="E12" t="s">
-        <v>102</v>
+        <v>86</v>
       </c>
       <c r="F12" t="s">
-        <v>103</v>
+        <v>87</v>
       </c>
       <c r="G12" t="s">
-        <v>104</v>
+        <v>88</v>
       </c>
       <c r="H12" t="s">
-        <v>102</v>
+        <v>86</v>
       </c>
       <c r="I12" t="s">
-        <v>101</v>
+        <v>85</v>
       </c>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>100</v>
+        <v>84</v>
       </c>
       <c r="B13" t="s">
-        <v>101</v>
+        <v>85</v>
       </c>
       <c r="C13" t="s">
-        <v>102</v>
+        <v>86</v>
       </c>
       <c r="D13" t="s">
-        <v>103</v>
+        <v>87</v>
       </c>
       <c r="E13" t="s">
-        <v>103</v>
+        <v>87</v>
       </c>
       <c r="F13" t="s">
-        <v>103</v>
+        <v>87</v>
       </c>
       <c r="G13" t="s">
-        <v>102</v>
+        <v>86</v>
       </c>
       <c r="H13" t="s">
-        <v>102</v>
+        <v>86</v>
       </c>
       <c r="I13" t="s">
-        <v>104</v>
+        <v>88</v>
       </c>
     </row>
     <row r="15" spans="1:12" ht="75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="B15" s="2"/>
-      <c r="C15" s="2"/>
-      <c r="D15" s="2"/>
-      <c r="E15" s="2"/>
-      <c r="F15" s="2"/>
-      <c r="G15" s="2"/>
-      <c r="H15" s="2"/>
-      <c r="I15" s="2"/>
+      <c r="A15" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="B15" s="7"/>
+      <c r="C15" s="7"/>
+      <c r="D15" s="7"/>
+      <c r="E15" s="7"/>
+      <c r="F15" s="7"/>
+      <c r="G15" s="7"/>
+      <c r="H15" s="7"/>
+      <c r="I15" s="7"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>